<commit_message>
Nuevos modelos sin biomasa constreñida, comparacion produccion de biomasa
</commit_message>
<xml_diff>
--- a/Data/HPLC_results/HPLC_results-processed_Juanjo_2.xlsx
+++ b/Data/HPLC_results/HPLC_results-processed_Juanjo_2.xlsx
@@ -1,25 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Proyectos\salmonella_metabolic_phoP_analysis\proteomics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\yannis\CNB\CNB\Data\HPLC_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDD4873A-91DA-4846-B0C1-9BBEB57A92D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F6021C-972C-4C50-A77E-142AB1402E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="06.11.25" sheetId="1" r:id="rId1"/>
     <sheet name="datos" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -380,13 +388,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -398,22 +403,22 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -459,7 +464,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -862,7 +869,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:M27"/>
+  <dimension ref="B3:M26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5546875" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="19.44140625" customWidth="1"/>
@@ -883,709 +890,706 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:13">
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="I3" s="2" t="s">
+      <c r="G3" s="27"/>
+      <c r="I3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="M3" s="2"/>
+      <c r="M3" s="1"/>
     </row>
     <row r="4" spans="2:13" ht="28.8">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="10" t="s">
+      <c r="K4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="L4" s="10" t="s">
+      <c r="L4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="M4" s="11" t="s">
+      <c r="M4" s="10" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="2:13">
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>1</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="12">
         <v>0</v>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="13">
         <v>0.02</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="14">
         <v>31.310951541023801</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="15">
         <v>5.6409810296308498</v>
       </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" spans="2:13">
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>2</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="12">
         <v>5.33</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <v>0.151</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="14">
         <v>23.858350949006802</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="15">
         <v>4.2983205069730701</v>
       </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="19">
+      <c r="H6" s="8"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="18">
         <v>0.15667318344737699</v>
       </c>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
     </row>
     <row r="7" spans="2:13">
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>3</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="12">
         <v>6.58</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <v>0.36499999999999999</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="14">
         <v>22.202016683774101</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="15">
         <v>3.9999153257487499</v>
       </c>
-      <c r="H7" s="9"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="19">
+      <c r="H7" s="8"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="18">
         <v>0.32936787227109798</v>
       </c>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
     </row>
     <row r="8" spans="2:13">
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>4</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="12">
         <v>7.33</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="17">
         <v>0.59199999999999997</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="14">
         <v>20.9177049666316</v>
       </c>
-      <c r="G8" s="16">
+      <c r="G8" s="15">
         <v>3.7685337267883399</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H8" s="8">
         <v>34.200000000000003</v>
       </c>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
     </row>
     <row r="9" spans="2:13">
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>5</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="12">
         <v>7.83</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="17">
         <v>0.78100000000000003</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="14">
         <v>18.1906573218874</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="15">
         <v>3.2772288231112299</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="8">
         <v>46</v>
       </c>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="19">
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="18">
         <v>0.74318344737699604</v>
       </c>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
     </row>
     <row r="10" spans="2:13">
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>6</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="12">
         <v>24.42</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="17">
         <v>1.61</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="14">
         <v>0</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="15">
         <v>0</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="8">
         <v>121</v>
       </c>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="19">
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="18">
         <v>0.78228413163897004</v>
       </c>
-      <c r="L10" s="19">
+      <c r="L10" s="18">
         <v>0.48491387843991302</v>
       </c>
-      <c r="M10" s="10">
+      <c r="M10" s="9">
         <v>225</v>
       </c>
     </row>
     <row r="11" spans="2:13">
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>7</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="12">
         <v>25.67</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="17">
         <v>1.65</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="14">
         <v>0</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="15">
         <v>0</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="8">
         <v>111</v>
       </c>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="19">
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="18">
         <v>0.51248941023134598</v>
       </c>
-      <c r="L11" s="19">
+      <c r="L11" s="18">
         <v>0.49243714116016601</v>
       </c>
-      <c r="M11" s="10">
+      <c r="M11" s="9">
         <v>217</v>
       </c>
     </row>
     <row r="12" spans="2:13">
-      <c r="B12" s="3">
+      <c r="B12" s="2">
         <v>8</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="12">
         <v>5.33</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="17">
         <v>0.11600000000000001</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="14">
         <v>25.495764015931599</v>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="15">
         <v>4.5933168451102304</v>
       </c>
-      <c r="H12" s="9"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="19">
+      <c r="H12" s="8"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="18">
         <v>0.117572499185402</v>
       </c>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
     </row>
     <row r="13" spans="2:13">
-      <c r="B13" s="3">
+      <c r="B13" s="2">
         <v>9</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="12">
         <v>6.58</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="17">
         <v>0.28399999999999997</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="14">
         <v>23.297399473737801</v>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="15">
         <v>4.1972594891885997</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="8">
         <v>17.100000000000001</v>
       </c>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="19">
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="18">
         <v>0.25116650374714899</v>
       </c>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
     </row>
     <row r="14" spans="2:13">
-      <c r="B14" s="3">
+      <c r="B14" s="2">
         <v>10</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="12">
         <v>7.33</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E14" s="17">
         <v>0.48199999999999998</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="14">
         <v>21.805346498762599</v>
       </c>
-      <c r="G14" s="16">
+      <c r="G14" s="15">
         <v>3.92845122521708</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H14" s="8">
         <v>28</v>
       </c>
-      <c r="I14" s="19">
+      <c r="I14" s="18">
         <v>0.150483507749371</v>
       </c>
-      <c r="J14" s="19">
+      <c r="J14" s="18">
         <v>0.22735156771180801</v>
       </c>
-      <c r="K14" s="19">
+      <c r="K14" s="18">
         <v>0.41082763115021198</v>
       </c>
-      <c r="L14" s="19">
+      <c r="L14" s="18">
         <v>0</v>
       </c>
-      <c r="M14" s="21">
+      <c r="M14" s="20">
         <v>7.5</v>
       </c>
     </row>
     <row r="15" spans="2:13">
-      <c r="B15" s="3">
+      <c r="B15" s="2">
         <v>11</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="12">
         <v>8.08</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="17">
         <v>0.76</v>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="14">
         <v>18.4534094054106</v>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="15">
         <v>3.32456623847877</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H15" s="8">
         <v>62</v>
       </c>
-      <c r="I15" s="19">
+      <c r="I15" s="18">
         <v>0.268379917869917</v>
       </c>
-      <c r="J15" s="19">
+      <c r="J15" s="18">
         <v>0.26737825216811201</v>
       </c>
-      <c r="K15" s="19">
+      <c r="K15" s="18">
         <v>0.72037471489084404</v>
       </c>
-      <c r="L15" s="19">
+      <c r="L15" s="18">
         <v>0</v>
       </c>
-      <c r="M15" s="21">
+      <c r="M15" s="20">
         <v>14.1</v>
       </c>
     </row>
     <row r="16" spans="2:13">
-      <c r="B16" s="3">
+      <c r="B16" s="2">
         <v>12</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="12">
         <v>24.42</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="17">
         <v>1.6</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="14">
         <v>0</v>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="15">
         <v>0</v>
       </c>
-      <c r="H16" s="9">
+      <c r="H16" s="8">
         <v>135</v>
       </c>
-      <c r="I16" s="19">
+      <c r="I16" s="18">
         <v>0.37832825539806603</v>
       </c>
-      <c r="J16" s="19">
+      <c r="J16" s="18">
         <v>0.173982655103402</v>
       </c>
-      <c r="K16" s="19">
+      <c r="K16" s="18">
         <v>0.808351254480287</v>
       </c>
-      <c r="L16" s="19">
+      <c r="L16" s="18">
         <v>0.46115620669174401</v>
       </c>
-      <c r="M16" s="21">
+      <c r="M16" s="20">
         <v>218</v>
       </c>
     </row>
     <row r="17" spans="2:13">
-      <c r="B17" s="3">
+      <c r="B17" s="2">
         <v>13</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D17" s="13">
+      <c r="D17" s="12">
         <v>25.67</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="17">
         <v>1.6379999999999999</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="14">
         <v>0</v>
       </c>
-      <c r="G17" s="16">
+      <c r="G17" s="15">
         <v>0</v>
       </c>
-      <c r="H17" s="9">
+      <c r="H17" s="8">
         <v>158</v>
       </c>
-      <c r="I17" s="19">
+      <c r="I17" s="18">
         <v>0.36110743144787399</v>
       </c>
-      <c r="J17" s="19">
+      <c r="J17" s="18">
         <v>0.18398932621747799</v>
       </c>
-      <c r="K17" s="19">
+      <c r="K17" s="18">
         <v>0.52878136200716797</v>
       </c>
-      <c r="L17" s="19">
+      <c r="L17" s="18">
         <v>0.46966937240150503</v>
       </c>
-      <c r="M17" s="21">
+      <c r="M17" s="20">
         <v>231</v>
       </c>
     </row>
     <row r="18" spans="2:13">
-      <c r="B18" s="3">
+      <c r="B18" s="2">
         <v>14</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="13">
+      <c r="D18" s="12">
         <v>8.08</v>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="17">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="14">
         <v>25.080521009105698</v>
       </c>
-      <c r="G18" s="16">
+      <c r="G18" s="15">
         <v>4.5185066650004702</v>
       </c>
-      <c r="H18" s="9">
+      <c r="H18" s="8">
         <v>115</v>
       </c>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="21"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="20"/>
     </row>
     <row r="19" spans="2:13">
-      <c r="B19" s="3">
+      <c r="B19" s="2">
         <v>15</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="13">
+      <c r="D19" s="12">
         <v>16</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="17">
         <v>0.26</v>
       </c>
-      <c r="F19" s="15">
+      <c r="F19" s="14">
         <v>24.474454777917</v>
       </c>
-      <c r="G19" s="16">
+      <c r="G19" s="15">
         <v>4.4093177727895299</v>
       </c>
-      <c r="H19" s="9"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="21"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="18"/>
+      <c r="M19" s="20"/>
     </row>
     <row r="20" spans="2:13">
-      <c r="B20" s="3">
+      <c r="B20" s="2">
         <v>16</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="12">
         <v>18.25</v>
       </c>
-      <c r="E20" s="18">
+      <c r="E20" s="17">
         <v>0.38300000000000001</v>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="14">
         <v>23.767032760625099</v>
       </c>
-      <c r="G20" s="16">
+      <c r="G20" s="15">
         <v>4.2818686221542199</v>
       </c>
-      <c r="H20" s="9"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="21">
+      <c r="H20" s="8"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
+      <c r="L20" s="18"/>
+      <c r="M20" s="20">
         <v>16</v>
       </c>
     </row>
     <row r="21" spans="2:13">
-      <c r="B21" s="3">
+      <c r="B21" s="2">
         <v>17</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="13">
+      <c r="D21" s="12">
         <v>22.33</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="17">
         <v>0.65700000000000003</v>
       </c>
-      <c r="F21" s="15">
+      <c r="F21" s="14">
         <v>21.462739990849801</v>
       </c>
-      <c r="G21" s="16">
+      <c r="G21" s="15">
         <v>3.8667272367515002</v>
       </c>
-      <c r="H21" s="9"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="19"/>
-      <c r="L21" s="19"/>
-      <c r="M21" s="21">
+      <c r="H21" s="8"/>
+      <c r="I21" s="18"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18"/>
+      <c r="L21" s="18"/>
+      <c r="M21" s="20">
         <v>36</v>
       </c>
     </row>
     <row r="22" spans="2:13">
-      <c r="B22" s="3">
+      <c r="B22" s="2">
         <v>18</v>
       </c>
-      <c r="C22" s="22" t="s">
+      <c r="C22" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="D22" s="13">
+      <c r="D22" s="12">
         <v>24.42</v>
       </c>
-      <c r="E22" s="18">
+      <c r="E22" s="17">
         <v>1.02</v>
       </c>
-      <c r="F22" s="15">
+      <c r="F22" s="14">
         <v>16.5739291092694</v>
       </c>
-      <c r="G22" s="16">
+      <c r="G22" s="15">
         <v>2.9859590683259798</v>
       </c>
-      <c r="H22" s="9">
+      <c r="H22" s="8">
         <v>26</v>
       </c>
-      <c r="I22" s="19">
+      <c r="I22" s="18">
         <v>0.29752285070870299</v>
       </c>
-      <c r="J22" s="19">
+      <c r="J22" s="18">
         <v>0.23002001334222799</v>
       </c>
-      <c r="K22" s="19">
+      <c r="K22" s="18">
         <v>0.28766047572499198</v>
       </c>
-      <c r="L22" s="19">
+      <c r="L22" s="18">
         <v>0</v>
       </c>
-      <c r="M22" s="21">
+      <c r="M22" s="20">
         <v>62.3</v>
       </c>
     </row>
     <row r="23" spans="2:13">
-      <c r="B23" s="3">
+      <c r="B23" s="2">
         <v>19</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="C23" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="12">
         <v>28.33</v>
       </c>
-      <c r="E23" s="18">
+      <c r="E23" s="17">
         <v>1.4139999999999999</v>
       </c>
-      <c r="F23" s="15">
+      <c r="F23" s="14">
         <v>9.7241287188137502</v>
       </c>
-      <c r="G23" s="16">
+      <c r="G23" s="15">
         <v>1.7518990299814901</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="8">
         <v>29</v>
       </c>
-      <c r="I23" s="19">
+      <c r="I23" s="18">
         <v>0.39819843687905698</v>
       </c>
-      <c r="J23" s="19">
+      <c r="J23" s="18">
         <v>0.40747164776517703</v>
       </c>
-      <c r="K23" s="19">
+      <c r="K23" s="18">
         <v>1.1374486803519099</v>
       </c>
-      <c r="L23" s="19">
+      <c r="L23" s="18">
         <v>0</v>
       </c>
-      <c r="M23" s="21">
+      <c r="M23" s="20">
         <v>154.4</v>
       </c>
     </row>
     <row r="24" spans="2:13">
-      <c r="B24" s="3">
+      <c r="B24" s="2">
         <v>20</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="13">
+      <c r="D24" s="12">
         <v>31.67</v>
       </c>
-      <c r="E24" s="18">
+      <c r="E24" s="17">
         <v>1.522</v>
       </c>
-      <c r="F24" s="23">
+      <c r="F24" s="22">
         <v>4.5216048047574997</v>
       </c>
-      <c r="G24" s="24">
+      <c r="G24" s="23">
         <v>0.81461232162511099</v>
       </c>
-      <c r="H24" s="9">
+      <c r="H24" s="8">
         <v>48.8</v>
       </c>
-      <c r="I24" s="25">
+      <c r="I24" s="24">
         <v>0.346535965028481</v>
       </c>
-      <c r="J24" s="25">
+      <c r="J24" s="24">
         <v>0.29339559706471002</v>
       </c>
-      <c r="K24" s="25">
+      <c r="K24" s="24">
         <v>1.79987943955686</v>
       </c>
-      <c r="L24" s="25">
+      <c r="L24" s="24">
         <v>7.2124331815482098E-2</v>
       </c>
-      <c r="M24" s="26">
+      <c r="M24" s="25">
         <v>197</v>
       </c>
     </row>
     <row r="26" spans="2:13">
-      <c r="C26" s="27"/>
-    </row>
-    <row r="27" spans="2:13">
-      <c r="C27" s="28"/>
+      <c r="C26" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1602,547 +1606,550 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="13">
+      <c r="D2" s="12">
         <v>0</v>
       </c>
-      <c r="E2" s="14">
+      <c r="E2" s="13">
         <v>0.02</v>
       </c>
-      <c r="F2" s="15">
+      <c r="F2" s="14">
         <v>31.310951541023801</v>
       </c>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="13">
+      <c r="D3" s="12">
         <v>5.33</v>
       </c>
-      <c r="E3" s="18">
+      <c r="E3" s="17">
         <v>0.151</v>
       </c>
-      <c r="F3" s="15">
+      <c r="F3" s="14">
         <v>23.858350949006802</v>
       </c>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="19">
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="18">
         <v>0.15667318344737699</v>
       </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="12">
         <v>6.58</v>
       </c>
-      <c r="E4" s="18">
+      <c r="E4" s="17">
         <v>0.36499999999999999</v>
       </c>
-      <c r="F4" s="15">
+      <c r="F4" s="14">
         <v>22.202016683774101</v>
       </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="19">
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="18">
         <v>0.32936787227109798</v>
       </c>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="12">
         <v>7.33</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="17">
         <v>0.59199999999999997</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="14">
         <v>20.9177049666316</v>
       </c>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="19"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="18">
+        <f>AVERAGE(I6,I4)</f>
+        <v>0.53627565982404701</v>
+      </c>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="12">
         <v>7.83</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <v>0.78100000000000003</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="14">
         <v>18.1906573218874</v>
       </c>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="19">
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="18">
         <v>0.74318344737699604</v>
       </c>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="12">
         <v>24.42</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <v>1.61</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="14">
         <v>0</v>
       </c>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="19">
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="18">
         <v>0.78228413163897004</v>
       </c>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="3">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="12">
         <v>25.67</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="17">
         <v>1.65</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="14">
         <v>0</v>
       </c>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="19">
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="18">
         <v>0.51248941023134598</v>
       </c>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="3">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="12">
         <v>5.33</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="17">
         <v>0.11600000000000001</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="14">
         <v>25.495764015931599</v>
       </c>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="19">
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="18">
         <v>0.117572499185402</v>
       </c>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="3">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="12">
         <v>6.58</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="17">
         <v>0.28399999999999997</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="14">
         <v>23.297399473737801</v>
       </c>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="19">
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="18">
         <v>0.25116650374714899</v>
       </c>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="3">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="12">
         <v>7.33</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="17">
         <v>0.48199999999999998</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="14">
         <v>21.805346498762599</v>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="18">
         <v>0.150483507749371</v>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="18">
         <v>0.22735156771180801</v>
       </c>
-      <c r="I11" s="19">
+      <c r="I11" s="18">
         <v>0.41082763115021198</v>
       </c>
     </row>
     <row r="12" spans="1:9">
-      <c r="A12" s="3">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="12">
         <v>8.08</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="17">
         <v>0.76</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="14">
         <v>18.4534094054106</v>
       </c>
-      <c r="G12" s="19">
+      <c r="G12" s="18">
         <v>0.268379917869917</v>
       </c>
-      <c r="H12" s="19">
+      <c r="H12" s="18">
         <v>0.26737825216811201</v>
       </c>
-      <c r="I12" s="19">
+      <c r="I12" s="18">
         <v>0.72037471489084404</v>
       </c>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" s="3">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="12">
         <v>24.42</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="17">
         <v>1.6</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="14">
         <v>0</v>
       </c>
-      <c r="G13" s="19">
+      <c r="G13" s="18">
         <v>0.37832825539806603</v>
       </c>
-      <c r="H13" s="19">
+      <c r="H13" s="18">
         <v>0.173982655103402</v>
       </c>
-      <c r="I13" s="19">
+      <c r="I13" s="18">
         <v>0.808351254480287</v>
       </c>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="3">
+      <c r="A14" s="2">
         <v>13</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="12">
         <v>25.67</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E14" s="17">
         <v>1.6379999999999999</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="14">
         <v>0</v>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="18">
         <v>0.36110743144787399</v>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="18">
         <v>0.18398932621747799</v>
       </c>
-      <c r="I14" s="19">
+      <c r="I14" s="18">
         <v>0.52878136200716797</v>
       </c>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15" s="3">
+      <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="C15" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="12">
         <v>8.08</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="17">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="14">
         <v>25.080521009105698</v>
       </c>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
     </row>
     <row r="16" spans="1:9">
-      <c r="A16" s="3">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="12">
         <v>16</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="17">
         <v>0.26</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="14">
         <v>24.474454777917</v>
       </c>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="3">
+      <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="13">
+      <c r="D17" s="12">
         <v>18.25</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="17">
         <v>0.38300000000000001</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="14">
         <v>23.767032760625099</v>
       </c>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
     </row>
     <row r="18" spans="1:9">
-      <c r="A18" s="3">
+      <c r="A18" s="2">
         <v>17</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="13">
+      <c r="D18" s="12">
         <v>22.33</v>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="17">
         <v>0.65700000000000003</v>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="14">
         <v>21.462739990849801</v>
       </c>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="3">
+      <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="13">
+      <c r="D19" s="12">
         <v>24.42</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="17">
         <v>1.02</v>
       </c>
-      <c r="F19" s="15">
+      <c r="F19" s="14">
         <v>16.5739291092694</v>
       </c>
-      <c r="G19" s="19">
+      <c r="G19" s="18">
         <v>0.29752285070870299</v>
       </c>
-      <c r="H19" s="19">
+      <c r="H19" s="18">
         <v>0.23002001334222799</v>
       </c>
-      <c r="I19" s="19">
+      <c r="I19" s="18">
         <v>0.28766047572499198</v>
       </c>
     </row>
     <row r="20" spans="1:9">
-      <c r="A20" s="3">
+      <c r="A20" s="2">
         <v>19</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="12">
         <v>28.33</v>
       </c>
-      <c r="E20" s="18">
+      <c r="E20" s="17">
         <v>1.4139999999999999</v>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="14">
         <v>9.7241287188137502</v>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="18">
         <v>0.39819843687905698</v>
       </c>
-      <c r="H20" s="19">
+      <c r="H20" s="18">
         <v>0.40747164776517703</v>
       </c>
-      <c r="I20" s="19">
+      <c r="I20" s="18">
         <v>1.1374486803519099</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15" thickBot="1">
-      <c r="A21" s="3">
+      <c r="A21" s="2">
         <v>20</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="13">
+      <c r="D21" s="12">
         <v>31.67</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="17">
         <v>1.522</v>
       </c>
-      <c r="F21" s="23">
+      <c r="F21" s="22">
         <v>4.5216048047574997</v>
       </c>
-      <c r="G21" s="25">
+      <c r="G21" s="24">
         <v>0.346535965028481</v>
       </c>
-      <c r="H21" s="25">
+      <c r="H21" s="24">
         <v>0.29339559706471002</v>
       </c>
-      <c r="I21" s="25">
+      <c r="I21" s="24">
         <v>1.79987943955686</v>
       </c>
     </row>

</xml_diff>